<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-02 Le cheval de bois sous la haie
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-02.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-02.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chemin du village puis véranda</t>
+          <t>chemin du village puis véranda, haie de buis, poussière, abeille</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Victorino, maman</t>
+          <t>Amir, Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir cherche son cheval de bois sous la haie. Victorino l'aide. Un rire commence. Maman dit : le corps n'est pas une blague. Sur la véranda, ils font une écurie d'argile.</t>
+          <t>Le chemin du village sent la poussière chaude. La haie de buis pique. Une abeille va d'une fleur à l'autre. Sur une feuille, un éclat de buis brille. Amir veut son cheval de bois, maintenant, sous la haie. Il écarte trop vite : le bois glisse, l'éclat saute. Victorino s'agenouille lentement. Un petit rire commence, puis s'arrête. Ils cherchent ensemble. Merci vécu. Sur la véranda, l'écurie d'argile s'affaisse. Amir refuse de foncer. L'éclat de buis tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La poussière du chemin sent encore le soleil. La haie de buis est chaude et serrée. Une abeille va d'une fleur à l'autre. Le portail de fer est tiède. Un caillou blanc brille dans l'ornière. Tu as vu le portail, Amir ? Il est chaud. Oui. Le soleil l'a touché. En ce moment, Amir cherche dans l'herbe. L'herbe est sèche et un peu piquante. Mon cheval de bois. Il a roulé. Regarde sous la haie. Victorino arrive près du portail. Ses genoux ont déjà de la poussière. Victorino a un corps plus rond. Amir a un corps plus mince. Les corps ont des formes différentes. Un petit rire commence. Le corps n'est pas une blague. On joue. Amir ferme la bouche. On cherche le cheval ? On cherche. Ils écartent une branche. Les feuilles sentent le vert. Un caillou roule. Pas lui. Le bois du cheval apparaît. Te voilà. Il a de la terre au nez. On va le laver à la maison.</t>
+          <t>Le chemin du village sent la poussière chaude. La haie de buis est serrée, un peu piquante. Une abeille va d'une fleur à l'autre. Le portail de fer est tiède sous la main. Tu as vu le portail, Amir ? Il est chaud. Le soleil l'a touché. La haie aussi. Elle pique un peu. La poussière colle aux orteils. Le buis sent le vert chaud. Une feuille tremble au bord de la haie. Sur la feuille, un éclat de buis brille. Il brille, papa. Tu le vois, sur la feuille ? Oui, il brille. C'est petit, cet éclat. L'herbe est sèche, un peu dure. Mon cheval de bois. Il a roulé. Sous la haie ? Oui, maman. Je le veux, maintenant ! On le cherche ? Oui, papa. En ce moment, Amir cherche dans l'herbe. Les tiges piquent ses paumes. Il écarte une branche trop vite. Le bois glisse plus loin, sous les feuilles. Il est parti ! L'éclat de buis saute près du portail. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le cheval ? Oui, papa. Tes genoux sont dans l'herbe ? Oui, maman. Victorino arrive près du portail. Il prend son temps, les pieds dans la poussière. J'aide. Vite ! Victorino s'agenouille plus lentement. Un petit rire commence, chez Amir. Victorino baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Amir ferme la bouche. Ses joues sont chaudes, un peu. On cherche le cheval ? Victorino ne répond pas tout de suite. On cherche. Tu tiens la branche, Amir ? Oui.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La poussière du chemin sent encore le soleil. La haie de buis est chaude et serrée. Une abeille va d'une fleur à l'autre. Le portail de fer est tiède. Un caillou blanc brille dans l'ornière. Tu as vu le portail, Amir ? Il est chaud. Oui. Le soleil l'a touché. En ce moment, Amir cherche dans l'herbe. L'herbe est sèche et un peu piquante. Mon cheval de bois. Il a roulé. Regarde sous la haie. Victorino arrive près du portail. Ses genoux ont déjà de la poussière. Victorino a un corps plus rond. Amir a un corps plus mince. Les corps ont des formes différentes. Un petit rire commence. Le corps n'est pas une blague. On joue. Amir ferme la bouche. On cherche le cheval ? On cherche. Ils écartent une branche. Les feuilles sentent le vert. Un caillou roule. Pas lui. Le bois du cheval apparaît. Te voilà. Il a de la terre au nez. On va le laver à la maison.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le chemin du village sent la poussière chaude. La haie de buis est serrée, un peu piquante. Une abeille va d'une fleur à l'autre. Le portail de fer est tiède sous la main. Tu as vu le portail, Amir ? Il est chaud. Le soleil l'a touché. La haie aussi. Elle pique un peu. La poussière colle aux orteils. Le buis sent le vert chaud. Une feuille tremble au bord de la haie. Sur la feuille, un &lt;emphasis level="moderate"&gt;éclat de buis&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la feuille ? Oui, il brille. C'est petit, cet éclat. L'herbe est sèche, un peu dure. Mon cheval de bois. Il a roulé. Sous la haie ? Oui, maman. Je le veux, maintenant ! On le cherche ? Oui, papa. En ce moment, Amir cherche dans l'herbe. Les tiges piquent ses paumes. Il écarte une branche trop vite. Le bois glisse plus loin, sous les feuilles. Il est parti ! L'éclat de buis saute près du portail. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le cheval ? Oui, papa. Tes genoux sont dans l'herbe ? Oui, maman. Victorino arrive près du portail. Il prend son temps, les pieds dans la poussière. J'aide. Vite ! Victorino s'agenouille plus lentement. Un petit rire commence, chez Amir. Victorino baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Amir ferme la bouche. Ses joues sont chaudes, un peu. On cherche le cheval ? Victorino ne répond pas tout de suite. On cherche. Tu tiens la branche, Amir ? Oui.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nora est au parc avec maman. Lila arrive. Elles n'ont pas la même taille. Lila est plus petite. Nora est plus grande. Les tailles sont différentes. Les &lt;emphasis&gt;corps&lt;/emphasis&gt; ont des formes différentes. Un petit rire commence. Maman parle tout de suite. Maman dit : le corps n'est pas une blague. On joue ensemble. Nora ferme la bouche. Elle tend le ballon. Elles jouent. Le ballon est doux. Plus tard, elles rentrent en classe. Sur la table, il y a de la pâte. Les tabliers tombent différemment. Encore un petit rire. Nora dit : le corps n'est pas une blague. On joue ensemble. Elles font des formes. La pâte est froide. Au parc, puis en classe, c'est pareil. On joue. On ne commente pas le corps pour rabaisser. L'amitié ne dépend pas de la forme. [pause]</t>
+          <t>Le chemin du village sent la poussière chaude. La haie de buis est serrée, un peu piquante. Une abeille va d'une fleur à l'autre. Le portail de fer est tiède sous la main. Tu as vu le portail, Amir ? Il est chaud. Le soleil l'a touché. La haie aussi. Elle pique un peu. La poussière colle aux orteils. Le buis sent le vert chaud. Une feuille tremble au bord de la haie. Sur la feuille, un &lt;emphasis&gt;éclat de buis&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la feuille ? Oui, il brille. C'est petit, cet éclat. L'herbe est sèche, un peu dure. Mon cheval de bois. Il a roulé. Sous la haie ? Oui, maman. Je le veux, maintenant ! On le cherche ? Oui, papa. En ce moment, Amir cherche dans l'herbe. Les tiges piquent ses paumes. Il écarte une branche trop vite. Le bois glisse plus loin, sous les feuilles. Il est parti ! L'éclat de buis saute près du portail. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le cheval ? Oui, papa. Tes genoux sont dans l'herbe ? Oui, maman. Victorino arrive près du portail. Il prend son temps, les pieds dans la poussière. J'aide. Vite ! Victorino s'agenouille plus lentement. Un petit rire commence, chez Amir. Victorino baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Amir ferme la bouche. Ses joues sont chaudes, un peu. On cherche le cheval ? Victorino ne répond pas tout de suite. On cherche. Tu tiens la branche, Amir ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de buis</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,47 +1326,73 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=il_veut_le_cheval_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La poussière du chemin sent encore le soleil.
-narrateur|La haie de buis est chaude et serrée.
+          <t>narrateur|Le chemin du village sent la poussière chaude.
+narrateur|La haie de buis est serrée, un peu piquante.
 narrateur|Une abeille va d'une fleur à l'autre.
-narrateur|Le portail de fer est tiède.
-narrateur|Un caillou blanc brille dans l'ornière.
-maman|Tu as vu le portail, Amir ?
+narrateur|Le portail de fer est tiède sous la main.
+papa|Tu as vu le portail, Amir ?
 enfant-m|Il est chaud.
-maman|Oui.
-maman|Le soleil l'a touché.
-narrateur|En ce moment, Amir cherche dans l'herbe.
-narrateur|L'herbe est sèche et un peu piquante.
+papa|Le soleil l'a touché.
+maman|La haie aussi.
+enfant-m|Elle pique un peu.
+narrateur|La poussière colle aux orteils.
+narrateur|Le buis sent le vert chaud.
+narrateur|Une feuille tremble au bord de la haie.
+narrateur|Sur la feuille, un éclat de buis brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur la feuille ?
+enfant-m|Oui, il brille.
+maman|C'est petit, cet éclat.
+narrateur|L'herbe est sèche, un peu dure.
 enfant-m|Mon cheval de bois.
 enfant-m|Il a roulé.
-maman|Regarde sous la haie.
+maman|Sous la haie ?
+enfant-m|Oui, maman.
+enfant-m|Je le veux, maintenant !
+papa|On le cherche ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Amir cherche dans l'herbe.
+narrateur|Les tiges piquent ses paumes.
+narrateur|Il écarte une branche trop vite.
+narrateur|Le bois glisse plus loin, sous les feuilles.
+enfant-m|Il est parti !
+narrateur|L'éclat de buis saute près du portail.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le cheval ?
+enfant-m|Oui, papa.
+maman|Tes genoux sont dans l'herbe ?
+enfant-m|Oui, maman.
 narrateur|Victorino arrive près du portail.
-narrateur|Ses genoux ont déjà de la poussière.
-narrateur|Victorino a un corps plus rond.
-narrateur|Amir a un corps plus mince.
-narrateur|Les corps ont des formes différentes.
-narrateur|Un petit rire commence.
-maman|Le corps n'est pas une blague.
-maman|On joue.
+narrateur|Il prend son temps, les pieds dans la poussière.
+copain|J'aide.
+enfant-m|Vite !
+narrateur|Victorino s'agenouille plus lentement.
+narrateur|Un petit rire commence, chez Amir.
+narrateur|Victorino baisse les yeux.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Le rire s'arrête net.
 narrateur|Amir ferme la bouche.
+narrateur|Ses joues sont chaudes, un peu.
 enfant-m|On cherche le cheval ?
+narrateur|Victorino ne répond pas tout de suite.
 copain|On cherche.
-narrateur|Ils écartent une branche.
-narrateur|Les feuilles sentent le vert.
-narrateur|Un caillou roule.
-enfant-m|Pas lui.
-narrateur|Le bois du cheval apparaît.
-enfant-m|Te voilà.
-copain|Il a de la terre au nez.
-maman|On va le laver à la maison.</t>
+papa|Tu tiens la branche, Amir ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>abeille,chemin,haie</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1424,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps n'est pas une &lt;emphasis level="moderate"&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps n'est pas une &lt;emphasis&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1428,7 +1454,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On joue. Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>On joue. Que fait Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1466,18 +1492,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1492,38 +1518,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>blague</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1532,23 +1558,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_rire_s_est_arrete_ils_cherchent_ensemble; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1581,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sur la véranda, l'argile attend. Elle est froide et un peu grise. Amir lave le cheval. L'eau fait un filet brun. Le bois redevient lisse. Il est propre. Il a besoin d'une écurie. On la fait. Ils pressent l'argile. Ça fait un bruit mou. Amir dresse un mur. Victorino dresse l'autre mur. Un mur s'affaisse. Il est fatigué. On le tient ensemble. Victorino appuie tout doux. Amir pose un toit plat. Le cheval entre dans l'écurie. Sa jambe de bois touche l'argile. Il est à la maison. Bravo, Amir. Tu as trouvé le cheval. Vous jouez. L'amitié ne dépend pas de la forme.</t>
+          <t>Amir tend une branche vers Victorino. Victorino la prend, sans se presser. Tu tiens ? Oui. Ils écartent les feuilles, ensemble. Les feuilles sentent le vert. Un caillou roule. Pas lui. Plus bas. Le bois du cheval apparaît. Te voilà. Il a de la terre au nez. On le lave, sur la véranda ? Oui, maman. Je pousse le portail. La véranda est à l'ombre, un peu froide. Un bac d'eau attend près du banc. Amir lave le cheval. L'eau fait un filet brun. Il est propre. Il a besoin d'une écurie ? Oui, maintenant ! On la fait. L'argile attend sur une planche. Elle est froide, un peu grise. Amir dresse un mur trop vite. Le mur s'affaisse, mou. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Personne ne dit la suite. Il écoute l'abeille, près de la haie. Attends. Victorino appuie de l'autre côté. Les deux murs tiennent, un peu. Un toit ? Pas trop vite. Amir pose un toit plat. Le cheval entre dans l'écurie. Sa jambe de bois touche l'argile. Il est à la maison. Merci, Amir. Papa a vu les deux mains sur l'argile. Victorino, tu as vu le cheval ? Oui. Il tient. Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sur la véranda, l'argile attend. Elle est froide et un peu grise. Amir lave le cheval. L'eau fait un filet brun. Le bois redevient lisse. Il est propre. Il a besoin d'une écurie. On la fait. Ils pressent l'argile. Ça fait un bruit mou. Amir dresse un mur. Victorino dresse l'autre mur. Un mur s'affaisse. Il est fatigué. On le tient ensemble. Victorino appuie tout doux. Amir pose un toit plat. Le cheval entre dans l'écurie. Sa jambe de bois touche l'argile. Il est à la maison. Bravo, Amir. Tu as trouvé le cheval. Vous jouez. L'amitié ne dépend pas de la forme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend une branche vers Victorino. Victorino la prend, sans se presser. Tu tiens ? Oui. Ils écartent les feuilles, ensemble. Les feuilles sentent le vert. Un caillou roule. Pas lui. Plus bas. Le bois du cheval apparaît. Te voilà. Il a de la terre au nez. On le lave, sur la véranda ? Oui, maman. Je pousse le portail. La véranda est à l'ombre, un peu froide. Un bac d'eau attend près du banc. Amir lave le cheval. L'eau fait un filet brun. Il est propre. Il a besoin d'une &lt;emphasis level="moderate"&gt;écurie&lt;/emphasis&gt; ? Oui, maintenant ! On la fait. L'argile attend sur une planche. Elle est froide, un peu grise. Amir dresse un mur trop vite. Le mur s'affaisse, mou. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Personne ne dit la suite. Il écoute l'abeille, près de la haie. Attends. Victorino appuie de l'autre côté. Les deux murs tiennent, un peu. Un toit ? Pas trop vite. Amir pose un toit plat. Le cheval entre dans l'écurie. Sa jambe de bois touche l'argile. Il est à la maison. Merci, Amir. Papa a vu les deux mains sur l'argile. Victorino, tu as vu le cheval ? Oui. Il tient. Le ventre d'Amir se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nora a entendu maman. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Nora et Lila ont joué. Deux fois. [pause]</t>
+          <t>Amir tend une branche vers Victorino. Victorino la prend, sans se presser. Tu tiens ? Oui. Ils écartent les feuilles, ensemble. Les feuilles sentent le vert. Un caillou roule. Pas lui. Plus bas. Le bois du cheval apparaît. Te voilà. Il a de la terre au nez. On le lave, sur la véranda ? Oui, maman. Je pousse le portail. La véranda est à l'ombre, un peu froide. Un bac d'eau attend près du banc. Amir lave le cheval. L'eau fait un filet brun. Il est propre. Il a besoin d'une &lt;emphasis&gt;écurie&lt;/emphasis&gt; ? Oui, maintenant ! On la fait. L'argile attend sur une planche. Elle est froide, un peu grise. Amir dresse un mur trop vite. Le mur s'affaisse, mou. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Personne ne dit la suite. Il écoute l'abeille, près de la haie. Attends. Victorino appuie de l'autre côté. Les deux murs tiennent, un peu. Un toit ? Pas trop vite. Amir pose un toit plat. Le cheval entre dans l'écurie. Sa jambe de bois touche l'argile. Il est à la maison. Merci, Amir. Papa a vu les deux mains sur l'argile. Victorino, tu as vu le cheval ? Oui. Il tient. Le ventre d'Amir se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1638,7 +1664,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1646,10 +1672,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1672,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>écurie</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,35 +1746,64 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_la_branche_puis_l_argile; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sur la véranda, l'argile attend.
-narrateur|Elle est froide et un peu grise.
+          <t>narrateur|Amir tend une branche vers Victorino.
+narrateur|Victorino la prend, sans se presser.
+enfant-m|Tu tiens ?
+copain|Oui.
+narrateur|Ils écartent les feuilles, ensemble.
+narrateur|Les feuilles sentent le vert.
+narrateur|Un caillou roule.
+enfant-m|Pas lui.
+copain|Plus bas.
+narrateur|Le bois du cheval apparaît.
+enfant-m|Te voilà.
+copain|Il a de la terre au nez.
+maman|On le lave, sur la véranda ?
+enfant-m|Oui, maman.
+papa|Je pousse le portail.
+narrateur|La véranda est à l'ombre, un peu froide.
+narrateur|Un bac d'eau attend près du banc.
 narrateur|Amir lave le cheval.
 narrateur|L'eau fait un filet brun.
-narrateur|Le bois redevient lisse.
 enfant-m|Il est propre.
-maman|Il a besoin d'une écurie.
+papa|Il a besoin d'une écurie ?
+enfant-m|Oui, maintenant !
 copain|On la fait.
-narrateur|Ils pressent l'argile.
-narrateur|Ça fait un bruit mou.
-narrateur|Amir dresse un mur.
-narrateur|Victorino dresse l'autre mur.
-narrateur|Un mur s'affaisse.
-enfant-m|Il est fatigué.
-maman|On le tient ensemble.
-narrateur|Victorino appuie tout doux.
+narrateur|L'argile attend sur une planche.
+narrateur|Elle est froide, un peu grise.
+narrateur|Amir dresse un mur trop vite.
+narrateur|Le mur s'affaisse, mou.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il pose les paumes à plat.
+narrateur|Personne ne dit la suite.
+narrateur|Il écoute l'abeille, près de la haie.
+copain|Attends.
+narrateur|Victorino appuie de l'autre côté.
+narrateur|Les deux murs tiennent, un peu.
+enfant-m|Un toit ?
+copain|Pas trop vite.
 narrateur|Amir pose un toit plat.
 narrateur|Le cheval entre dans l'écurie.
 narrateur|Sa jambe de bois touche l'argile.
 copain|Il est à la maison.
-maman|Bravo, Amir.
-maman|Tu as trouvé le cheval.
-maman|Vous jouez.
-maman|L'amitié ne dépend pas de la forme.</t>
+papa|Merci, Amir.
+narrateur|Papa a vu les deux mains sur l'argile.
+maman|Victorino, tu as vu le cheval ?
+copain|Oui.
+enfant-m|Il tient.
+narrateur|Le ventre d'Amir se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>eau,argile</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On laisse sécher ? Oui. L'argile devient un peu plus claire. Le cheval de bois attend dessous. Il dort. Tout petit. Tu as fini de presser l'argile ? Oui, maman. Ils se lavent les mains. L'eau est tiède. Dehors, le portail est encore chaud. Une abeille passe encore près de la haie. On le touchera demain. Merci, Victorino. Merci, Amir.</t>
+          <t>Amir veut le toit plus haut, d'un coup. Il pousse l'argile trop vite. Le toit glisse vers le bord. Ça tombe ! La jambe de bois s'enfonce un peu. Attends. Amir veut rattraper le toit, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la haie, par la véranda. L'éclat, papa ? Tu le vois, toi ? Sur la feuille. L'éclat de buis revient, sur la feuille. Le cheval, Amir ? Oui. Victorino tient le mur, sans parler. Amir pose le toit, plus lentement. La jambe de bois repose, droite. Il tient. Il dort. Tes mains sont propres ? Un peu d'argile, papa. L'eau est tiède. Ils se lavent les mains, près du bac. Dehors, le portail reste tiède. L'abeille est là. Près de la haie ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On laisse sécher ? Oui. L'argile devient un peu plus claire. Le cheval de bois attend dessous. Il dort. Tout petit. Tu as fini de presser l'argile ? Oui, maman. Ils se lavent les mains. L'eau est tiède. Dehors, le portail est encore chaud. Une abeille passe encore près de la haie. On le touchera demain. Merci, Victorino. Merci, Amir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut le toit plus haut, d'un coup. Il pousse l'argile trop vite. Le toit glisse vers le bord. Ça tombe ! La jambe de bois s'enfonce un peu. Attends. Amir veut rattraper le toit, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la haie, par la véranda. L'éclat, papa ? Tu le vois, toi ? Sur la feuille. L'&lt;emphasis level="moderate"&gt;éclat de buis&lt;/emphasis&gt; revient, sur la feuille. Le cheval, Amir ? Oui. Victorino tient le mur, sans parler. Amir pose le toit, plus lentement. La jambe de bois repose, droite. Il tient. Il dort. Tes mains sont propres ? Un peu d'argile, papa. L'eau est tiède. Ils se lavent les mains, près du bac. Dehors, le portail reste tiède. L'abeille est là. Près de la haie ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nora range un morceau de pâte. Lila range un emporte-pièce. Merci, dit maman. [pause]</t>
+          <t>Amir veut le toit plus haut, d'un coup. Il pousse l'argile trop vite. Le toit glisse vers le bord. Ça tombe ! La jambe de bois s'enfonce un peu. Attends. Amir veut rattraper le toit, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la haie, par la véranda. L'éclat, papa ? Tu le vois, toi ? Sur la feuille. L'&lt;emphasis&gt;éclat de buis&lt;/emphasis&gt; revient, sur la feuille. Le cheval, Amir ? Oui. Victorino tient le mur, sans parler. Amir pose le toit, plus lentement. La jambe de bois repose, droite. Il tient. Il dort. Tes mains sont propres ? Un peu d'argile, papa. L'eau est tiède. Ils se lavent les mains, près du bac. Dehors, le portail reste tiède. L'abeille est là. Près de la haie ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1887,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,10 +1895,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,28 +1919,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de buis</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,10 +1953,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,24 +1967,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_rattraper_le_toit_trop_vite; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On laisse sécher ?
+          <t>narrateur|Amir veut le toit plus haut, d'un coup.
+narrateur|Il pousse l'argile trop vite.
+narrateur|Le toit glisse vers le bord.
+enfant-m|Ça tombe !
+narrateur|La jambe de bois s'enfonce un peu.
+copain|Attends.
+narrateur|Amir veut rattraper le toit, d'un coup.
+narrateur|Amir refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde la haie, par la véranda.
+enfant-m|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-m|Sur la feuille.
+narrateur|L'éclat de buis revient, sur la feuille.
+maman|Le cheval, Amir ?
 enfant-m|Oui.
-narrateur|L'argile devient un peu plus claire.
-narrateur|Le cheval de bois attend dessous.
-copain|Il dort.
-enfant-m|Tout petit.
-maman|Tu as fini de presser l'argile ?
-enfant-m|Oui, maman.
-narrateur|Ils se lavent les mains.
-narrateur|L'eau est tiède.
-narrateur|Dehors, le portail est encore chaud.
-narrateur|Une abeille passe encore près de la haie.
-maman|On le touchera demain.
-enfant-m|Merci, Victorino.
-copain|Merci, Amir.</t>
+narrateur|Victorino tient le mur, sans parler.
+narrateur|Amir pose le toit, plus lentement.
+narrateur|La jambe de bois repose, droite.
+copain|Il tient.
+enfant-m|Il dort.
+papa|Tes mains sont propres ?
+enfant-m|Un peu d'argile, papa.
+maman|L'eau est tiède.
+narrateur|Ils se lavent les mains, près du bac.
+narrateur|Dehors, le portail reste tiède.
+enfant-m|L'abeille est là.
+papa|Près de la haie ?
+enfant-m|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>argile</t>
         </is>
       </c>
     </row>
@@ -1952,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a trouvé le cheval. On a fait l'écurie. Vous avez joué. La haie garde un peu de poussière.</t>
+          <t>Ils restent près de la planche. Le cheval de bois attend sous le toit. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. On est bien, ici. Dehors, le chemin sent la poussière. Une abeille passe près de la haie. Il est à la maison. Il est à la maison, Amir. Oui, maman. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Le nez a de la terre. Le nez du cheval porte une trace. La haie garde un peu de poussière. L'éclat de buis tient sur la feuille.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a trouvé le cheval. On a fait l'écurie. Vous avez joué. La haie garde un peu de poussière.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la planche. Le cheval de bois attend sous le toit. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. On est bien, ici. Dehors, le chemin sent la poussière. Une abeille passe près de la haie. Il est à la maison. Il est à la maison, Amir. Oui, maman. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Le nez a de la terre. Le nez du cheval porte une trace. La haie garde un peu de poussière. L'&lt;emphasis level="moderate"&gt;éclat de buis&lt;/emphasis&gt; tient sur la feuille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la planche. Le cheval de bois attend sous le toit. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. On est bien, ici. Dehors, le chemin sent la poussière. Une abeille passe près de la haie. Il est à la maison. Il est à la maison, Amir. Oui, maman. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Le nez a de la terre. Le nez du cheval porte une trace. La haie garde un peu de poussière. L'&lt;emphasis&gt;éclat de buis&lt;/emphasis&gt; tient sur la feuille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,7 +2093,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2017,10 +2101,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.12</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2127,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de buis</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,27 +2163,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_feuille; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|On a trouvé le cheval.
-copain|On a fait l'écurie.
-maman|Vous avez joué.
-narrateur|La haie garde un peu de poussière.</t>
+          <t>narrateur|Ils restent près de la planche.
+narrateur|Le cheval de bois attend sous le toit.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur la feuille ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|Dehors, le chemin sent la poussière.
+narrateur|Une abeille passe près de la haie.
+enfant-m|Il est à la maison.
+maman|Il est à la maison, Amir.
+enfant-m|Oui, maman.
+narrateur|Amir pose la joue près du bois.
+narrateur|Le bois est froid, un peu.
+enfant-m|C'est froid.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est froid.
+copain|Le nez a de la terre.
+narrateur|Le nez du cheval porte une trace.
+narrateur|La haie garde un peu de poussière.
+narrateur|L'éclat de buis tient sur la feuille.</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2309,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>